<commit_message>
pd css cross notebook + broader model
</commit_message>
<xml_diff>
--- a/outputs/pd_css_cross/Segments3_report.xlsx
+++ b/outputs/pd_css_cross/Segments3_report.xlsx
@@ -257,43 +257,43 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.5211267605633803</c:v>
+                  <c:v>0.8131868131868132</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.5189873417721519</c:v>
+                  <c:v>0.9047619047619048</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.6410256410256411</c:v>
+                  <c:v>0.9047619047619048</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.5689655172413793</c:v>
+                  <c:v>0.937888198757764</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.6949152542372882</c:v>
+                  <c:v>0.9182389937106918</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.7083333333333334</c:v>
+                  <c:v>0.9047619047619048</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.6341463414634146</c:v>
+                  <c:v>0.8873239436619719</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.6571428571428571</c:v>
+                  <c:v>0.8686131386861314</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.3928571428571428</c:v>
+                  <c:v>0.8625954198473282</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.6363636363636364</c:v>
+                  <c:v>0.881578947368421</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.5384615384615384</c:v>
+                  <c:v>0.8095238095238095</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.5526315789473685</c:v>
+                  <c:v>0.8222222222222222</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.6216216216216216</c:v>
+                  <c:v>0.8706896551724138</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -371,43 +371,43 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.1891891891891892</c:v>
+                  <c:v>0.3269230769230769</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.25</c:v>
+                  <c:v>0.4864864864864865</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.2166666666666667</c:v>
+                  <c:v>0.4943181818181818</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.2857142857142857</c:v>
+                  <c:v>0.4539473684210527</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.2352941176470588</c:v>
+                  <c:v>0.5135135135135135</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.1551724137931035</c:v>
+                  <c:v>0.4802631578947368</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.1964285714285714</c:v>
+                  <c:v>0.4901960784313725</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.2765957446808511</c:v>
+                  <c:v>0.4796747967479675</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.2549019607843137</c:v>
+                  <c:v>0.456</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.2916666666666667</c:v>
+                  <c:v>0.5528455284552846</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.375</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.3333333333333333</c:v>
+                  <c:v>0.5597014925373134</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.2380952380952381</c:v>
+                  <c:v>0.5357142857142857</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -485,43 +485,43 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.07692307692307693</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.08333333333333333</c:v>
+                  <c:v>0.07954545454545454</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.1739130434782609</c:v>
+                  <c:v>0.09174311926605505</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.2</c:v>
+                  <c:v>0.1458333333333333</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.1282051282051282</c:v>
+                  <c:v>0.1052631578947368</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.1627906976744186</c:v>
+                  <c:v>0.1395348837209302</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.16</c:v>
+                  <c:v>0.1458333333333333</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.09836065573770492</c:v>
+                  <c:v>0.1059602649006623</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.1857142857142857</c:v>
+                  <c:v>0.09580838323353294</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.180327868852459</c:v>
+                  <c:v>0.09659090909090909</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.07792207792207792</c:v>
+                  <c:v>0.1047120418848168</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.1267605633802817</c:v>
+                  <c:v>0.1170212765957447</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.07894736842105263</c:v>
+                  <c:v>0.07804878048780488</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -699,43 +699,43 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.5867768595041323</c:v>
+                  <c:v>0.4619289340101523</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.6030534351145038</c:v>
+                  <c:v>0.3809523809523809</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.484472049689441</c:v>
+                  <c:v>0.3402777777777778</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.3558282208588957</c:v>
+                  <c:v>0.3522975929978118</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.3959731543624161</c:v>
+                  <c:v>0.3613636363636364</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.3221476510067114</c:v>
+                  <c:v>0.3095823095823096</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.2789115646258503</c:v>
+                  <c:v>0.3234624145785877</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.2447552447552448</c:v>
+                  <c:v>0.3333333333333333</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.1879194630872483</c:v>
+                  <c:v>0.3096926713947991</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.2323943661971831</c:v>
+                  <c:v>0.3370288248337029</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.1925925925925926</c:v>
+                  <c:v>0.2923433874709977</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.2567567567567567</c:v>
+                  <c:v>0.2954048140043763</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.2387096774193548</c:v>
+                  <c:v>0.2516268980477224</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -813,43 +813,43 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.3057851239669421</c:v>
+                  <c:v>0.3959390862944163</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.3053435114503817</c:v>
+                  <c:v>0.4195011337868481</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.3726708074534161</c:v>
+                  <c:v>0.4074074074074074</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.4294478527607362</c:v>
+                  <c:v>0.3326039387308534</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.3422818791946309</c:v>
+                  <c:v>0.3363636363636364</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.3892617449664429</c:v>
+                  <c:v>0.3734643734643734</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.3809523809523809</c:v>
+                  <c:v>0.3485193621867881</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.3286713286713286</c:v>
+                  <c:v>0.2992700729927008</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.3422818791946309</c:v>
+                  <c:v>0.2955082742316785</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.3380281690140845</c:v>
+                  <c:v>0.2727272727272727</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.237037037037037</c:v>
+                  <c:v>0.2645011600928074</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.2635135135135135</c:v>
+                  <c:v>0.2932166301969366</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.2709677419354839</c:v>
+                  <c:v>0.3036876355748373</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -927,43 +927,43 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.1074380165289256</c:v>
+                  <c:v>0.1421319796954315</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.0916030534351145</c:v>
+                  <c:v>0.199546485260771</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.1428571428571428</c:v>
+                  <c:v>0.2523148148148148</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.2147239263803681</c:v>
+                  <c:v>0.3150984682713348</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.261744966442953</c:v>
+                  <c:v>0.3022727272727272</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.2885906040268457</c:v>
+                  <c:v>0.316953316953317</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.3401360544217687</c:v>
+                  <c:v>0.3280182232346242</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.4265734265734266</c:v>
+                  <c:v>0.3673965936739659</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.4697986577181208</c:v>
+                  <c:v>0.3947990543735225</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.4295774647887324</c:v>
+                  <c:v>0.3902439024390244</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.5703703703703704</c:v>
+                  <c:v>0.4431554524361949</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.4797297297297297</c:v>
+                  <c:v>0.4113785557986871</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.4903225806451613</c:v>
+                  <c:v>0.4446854663774403</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1141,43 +1141,43 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.5211267605633803</c:v>
+                  <c:v>0.8131868131868132</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.5189873417721519</c:v>
+                  <c:v>0.9047619047619048</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.6410256410256411</c:v>
+                  <c:v>0.9047619047619048</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.5689655172413793</c:v>
+                  <c:v>0.937888198757764</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.6949152542372882</c:v>
+                  <c:v>0.9182389937106918</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.7083333333333334</c:v>
+                  <c:v>0.9047619047619048</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.6341463414634146</c:v>
+                  <c:v>0.8873239436619719</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.6571428571428571</c:v>
+                  <c:v>0.8686131386861314</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.3928571428571428</c:v>
+                  <c:v>0.8625954198473282</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.6363636363636364</c:v>
+                  <c:v>0.881578947368421</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.5384615384615384</c:v>
+                  <c:v>0.8095238095238095</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.5526315789473685</c:v>
+                  <c:v>0.8222222222222222</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.6216216216216216</c:v>
+                  <c:v>0.8706896551724138</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1255,43 +1255,43 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.1891891891891892</c:v>
+                  <c:v>0.3269230769230769</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.25</c:v>
+                  <c:v>0.4864864864864865</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.2166666666666667</c:v>
+                  <c:v>0.4943181818181818</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.2857142857142857</c:v>
+                  <c:v>0.4539473684210527</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.2352941176470588</c:v>
+                  <c:v>0.5135135135135135</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.1551724137931035</c:v>
+                  <c:v>0.4802631578947368</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.1964285714285714</c:v>
+                  <c:v>0.4901960784313725</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.2765957446808511</c:v>
+                  <c:v>0.4796747967479675</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.2549019607843137</c:v>
+                  <c:v>0.456</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.2916666666666667</c:v>
+                  <c:v>0.5528455284552846</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.375</c:v>
+                  <c:v>0.5</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.3333333333333333</c:v>
+                  <c:v>0.5597014925373134</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.2380952380952381</c:v>
+                  <c:v>0.5357142857142857</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1369,43 +1369,43 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.07692307692307693</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.08333333333333333</c:v>
+                  <c:v>0.07954545454545454</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.1739130434782609</c:v>
+                  <c:v>0.09174311926605505</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.2</c:v>
+                  <c:v>0.1458333333333333</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.1282051282051282</c:v>
+                  <c:v>0.1052631578947368</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.1627906976744186</c:v>
+                  <c:v>0.1395348837209302</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.16</c:v>
+                  <c:v>0.1458333333333333</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.09836065573770492</c:v>
+                  <c:v>0.1059602649006623</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.1857142857142857</c:v>
+                  <c:v>0.09580838323353294</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.180327868852459</c:v>
+                  <c:v>0.09659090909090909</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.07792207792207792</c:v>
+                  <c:v>0.1047120418848168</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.1267605633802817</c:v>
+                  <c:v>0.1170212765957447</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.07894736842105263</c:v>
+                  <c:v>0.07804878048780488</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1583,43 +1583,43 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.5867768595041323</c:v>
+                  <c:v>0.4619289340101523</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.6030534351145038</c:v>
+                  <c:v>0.3809523809523809</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.484472049689441</c:v>
+                  <c:v>0.3402777777777778</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.3558282208588957</c:v>
+                  <c:v>0.3522975929978118</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.3959731543624161</c:v>
+                  <c:v>0.3613636363636364</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.3221476510067114</c:v>
+                  <c:v>0.3095823095823096</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.2789115646258503</c:v>
+                  <c:v>0.3234624145785877</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.2447552447552448</c:v>
+                  <c:v>0.3333333333333333</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.1879194630872483</c:v>
+                  <c:v>0.3096926713947991</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.2323943661971831</c:v>
+                  <c:v>0.3370288248337029</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.1925925925925926</c:v>
+                  <c:v>0.2923433874709977</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.2567567567567567</c:v>
+                  <c:v>0.2954048140043763</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.2387096774193548</c:v>
+                  <c:v>0.2516268980477224</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1697,43 +1697,43 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.3057851239669421</c:v>
+                  <c:v>0.3959390862944163</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.3053435114503817</c:v>
+                  <c:v>0.4195011337868481</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.3726708074534161</c:v>
+                  <c:v>0.4074074074074074</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.4294478527607362</c:v>
+                  <c:v>0.3326039387308534</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.3422818791946309</c:v>
+                  <c:v>0.3363636363636364</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.3892617449664429</c:v>
+                  <c:v>0.3734643734643734</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.3809523809523809</c:v>
+                  <c:v>0.3485193621867881</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.3286713286713286</c:v>
+                  <c:v>0.2992700729927008</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.3422818791946309</c:v>
+                  <c:v>0.2955082742316785</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.3380281690140845</c:v>
+                  <c:v>0.2727272727272727</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.237037037037037</c:v>
+                  <c:v>0.2645011600928074</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.2635135135135135</c:v>
+                  <c:v>0.2932166301969366</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.2709677419354839</c:v>
+                  <c:v>0.3036876355748373</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1811,43 +1811,43 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.1074380165289256</c:v>
+                  <c:v>0.1421319796954315</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.0916030534351145</c:v>
+                  <c:v>0.199546485260771</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.1428571428571428</c:v>
+                  <c:v>0.2523148148148148</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.2147239263803681</c:v>
+                  <c:v>0.3150984682713348</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.261744966442953</c:v>
+                  <c:v>0.3022727272727272</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.2885906040268457</c:v>
+                  <c:v>0.316953316953317</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.3401360544217687</c:v>
+                  <c:v>0.3280182232346242</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.4265734265734266</c:v>
+                  <c:v>0.3673965936739659</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.4697986577181208</c:v>
+                  <c:v>0.3947990543735225</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.4295774647887324</c:v>
+                  <c:v>0.3902439024390244</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.5703703703703704</c:v>
+                  <c:v>0.4431554524361949</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.4797297297297297</c:v>
+                  <c:v>0.4113785557986871</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.4903225806451613</c:v>
+                  <c:v>0.4446854663774403</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1938,7 +1938,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>962025</xdr:colOff>
+      <xdr:colOff>1028700</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
@@ -1968,7 +1968,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>962025</xdr:colOff>
+      <xdr:colOff>1028700</xdr:colOff>
       <xdr:row>37</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
@@ -2003,7 +2003,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>962025</xdr:colOff>
+      <xdr:colOff>1028700</xdr:colOff>
       <xdr:row>21</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
@@ -2033,7 +2033,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>962025</xdr:colOff>
+      <xdr:colOff>1028700</xdr:colOff>
       <xdr:row>37</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
     </xdr:to>
@@ -2346,7 +2346,8 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="1" customWidth="1"/>
-    <col min="2" max="3" width="21.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="21.7109375" style="2" customWidth="1"/>
     <col min="5" max="5" width="20.7109375" style="2" customWidth="1"/>
     <col min="6" max="7" width="10.7109375" style="3" customWidth="1"/>
@@ -2402,22 +2403,22 @@
         <v>0</v>
       </c>
       <c r="B4" s="1">
-        <v>-0.5174374683146535</v>
+        <v>0.9502345014917034</v>
       </c>
       <c r="C4" s="1">
-        <v>3.203767666961591</v>
+        <v>8.014037340297495</v>
       </c>
       <c r="D4" s="2">
-        <v>0.5942947702060222</v>
+        <v>0.8767268862911796</v>
       </c>
       <c r="E4" s="2">
-        <v>0.3333333333333333</v>
+        <v>0.3334514528703048</v>
       </c>
       <c r="F4" s="3">
-        <v>631</v>
+        <v>1882</v>
       </c>
       <c r="G4" s="3">
-        <v>375</v>
+        <v>1650</v>
       </c>
       <c r="I4" s="1">
         <v>0</v>
@@ -2426,16 +2427,16 @@
         <v>8</v>
       </c>
       <c r="K4" s="2">
-        <v>0.5211267605633803</v>
+        <v>0.8131868131868132</v>
       </c>
       <c r="L4" s="2">
-        <v>0.5867768595041323</v>
+        <v>0.4619289340101523</v>
       </c>
       <c r="M4" s="3">
-        <v>71</v>
+        <v>182</v>
       </c>
       <c r="N4" s="3">
-        <v>37</v>
+        <v>148</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -2443,22 +2444,22 @@
         <v>1</v>
       </c>
       <c r="B5" s="1">
-        <v>-1.135530545938961</v>
+        <v>-1.043918035281563</v>
       </c>
       <c r="C5" s="1">
-        <v>-0.5181460438793203</v>
+        <v>0.9500194933372372</v>
       </c>
       <c r="D5" s="2">
-        <v>0.248811410459588</v>
+        <v>0.4848484848484849</v>
       </c>
       <c r="E5" s="2">
-        <v>0.3333333333333333</v>
+        <v>0.3332742735648476</v>
       </c>
       <c r="F5" s="3">
-        <v>631</v>
+        <v>1881</v>
       </c>
       <c r="G5" s="3">
-        <v>157</v>
+        <v>912</v>
       </c>
       <c r="I5" s="1">
         <v>0</v>
@@ -2467,16 +2468,16 @@
         <v>9</v>
       </c>
       <c r="K5" s="2">
-        <v>0.5189873417721519</v>
+        <v>0.9047619047619048</v>
       </c>
       <c r="L5" s="2">
-        <v>0.6030534351145038</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="M5" s="3">
-        <v>79</v>
+        <v>168</v>
       </c>
       <c r="N5" s="3">
-        <v>41</v>
+        <v>152</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -2484,22 +2485,22 @@
         <v>2</v>
       </c>
       <c r="B6" s="1">
-        <v>-2.435104178233598</v>
+        <v>-10.8317280747611</v>
       </c>
       <c r="C6" s="1">
-        <v>-1.136348485150166</v>
+        <v>-1.045108577584102</v>
       </c>
       <c r="D6" s="2">
-        <v>0.133122028526149</v>
+        <v>0.1052631578947368</v>
       </c>
       <c r="E6" s="2">
-        <v>0.3333333333333333</v>
+        <v>0.3332742735648476</v>
       </c>
       <c r="F6" s="3">
-        <v>631</v>
+        <v>1881</v>
       </c>
       <c r="G6" s="3">
-        <v>84</v>
+        <v>198</v>
       </c>
       <c r="I6" s="1">
         <v>0</v>
@@ -2508,16 +2509,16 @@
         <v>10</v>
       </c>
       <c r="K6" s="2">
-        <v>0.6410256410256411</v>
+        <v>0.9047619047619048</v>
       </c>
       <c r="L6" s="2">
-        <v>0.484472049689441</v>
+        <v>0.3402777777777778</v>
       </c>
       <c r="M6" s="3">
-        <v>78</v>
+        <v>147</v>
       </c>
       <c r="N6" s="3">
-        <v>50</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -2528,16 +2529,16 @@
         <v>11</v>
       </c>
       <c r="K7" s="2">
-        <v>0.5689655172413793</v>
+        <v>0.937888198757764</v>
       </c>
       <c r="L7" s="2">
-        <v>0.3558282208588957</v>
+        <v>0.3522975929978118</v>
       </c>
       <c r="M7" s="3">
-        <v>58</v>
+        <v>161</v>
       </c>
       <c r="N7" s="3">
-        <v>33</v>
+        <v>151</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -2548,16 +2549,16 @@
         <v>12</v>
       </c>
       <c r="K8" s="2">
-        <v>0.6949152542372882</v>
+        <v>0.9182389937106918</v>
       </c>
       <c r="L8" s="2">
-        <v>0.3959731543624161</v>
+        <v>0.3613636363636364</v>
       </c>
       <c r="M8" s="3">
-        <v>59</v>
+        <v>159</v>
       </c>
       <c r="N8" s="3">
-        <v>41</v>
+        <v>146</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -2568,16 +2569,16 @@
         <v>13</v>
       </c>
       <c r="K9" s="2">
-        <v>0.7083333333333334</v>
+        <v>0.9047619047619048</v>
       </c>
       <c r="L9" s="2">
-        <v>0.3221476510067114</v>
+        <v>0.3095823095823096</v>
       </c>
       <c r="M9" s="3">
-        <v>48</v>
+        <v>126</v>
       </c>
       <c r="N9" s="3">
-        <v>34</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -2588,16 +2589,16 @@
         <v>14</v>
       </c>
       <c r="K10" s="2">
-        <v>0.6341463414634146</v>
+        <v>0.8873239436619719</v>
       </c>
       <c r="L10" s="2">
-        <v>0.2789115646258503</v>
+        <v>0.3234624145785877</v>
       </c>
       <c r="M10" s="3">
-        <v>41</v>
+        <v>142</v>
       </c>
       <c r="N10" s="3">
-        <v>26</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -2608,16 +2609,16 @@
         <v>15</v>
       </c>
       <c r="K11" s="2">
-        <v>0.6571428571428571</v>
+        <v>0.8686131386861314</v>
       </c>
       <c r="L11" s="2">
-        <v>0.2447552447552448</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="M11" s="3">
-        <v>35</v>
+        <v>137</v>
       </c>
       <c r="N11" s="3">
-        <v>23</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -2628,16 +2629,16 @@
         <v>16</v>
       </c>
       <c r="K12" s="2">
-        <v>0.3928571428571428</v>
+        <v>0.8625954198473282</v>
       </c>
       <c r="L12" s="2">
-        <v>0.1879194630872483</v>
+        <v>0.3096926713947991</v>
       </c>
       <c r="M12" s="3">
-        <v>28</v>
+        <v>131</v>
       </c>
       <c r="N12" s="3">
-        <v>11</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -2648,16 +2649,16 @@
         <v>17</v>
       </c>
       <c r="K13" s="2">
-        <v>0.6363636363636364</v>
+        <v>0.881578947368421</v>
       </c>
       <c r="L13" s="2">
-        <v>0.2323943661971831</v>
+        <v>0.3370288248337029</v>
       </c>
       <c r="M13" s="3">
-        <v>33</v>
+        <v>152</v>
       </c>
       <c r="N13" s="3">
-        <v>21</v>
+        <v>134</v>
       </c>
     </row>
     <row r="14" spans="1:14">
@@ -2668,16 +2669,16 @@
         <v>18</v>
       </c>
       <c r="K14" s="2">
-        <v>0.5384615384615384</v>
+        <v>0.8095238095238095</v>
       </c>
       <c r="L14" s="2">
-        <v>0.1925925925925926</v>
+        <v>0.2923433874709977</v>
       </c>
       <c r="M14" s="3">
-        <v>26</v>
+        <v>126</v>
       </c>
       <c r="N14" s="3">
-        <v>14</v>
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:14">
@@ -2688,16 +2689,16 @@
         <v>19</v>
       </c>
       <c r="K15" s="2">
-        <v>0.5526315789473685</v>
+        <v>0.8222222222222222</v>
       </c>
       <c r="L15" s="2">
-        <v>0.2567567567567567</v>
+        <v>0.2954048140043763</v>
       </c>
       <c r="M15" s="3">
-        <v>38</v>
+        <v>135</v>
       </c>
       <c r="N15" s="3">
-        <v>21</v>
+        <v>111</v>
       </c>
     </row>
     <row r="16" spans="1:14">
@@ -2708,16 +2709,16 @@
         <v>20</v>
       </c>
       <c r="K16" s="2">
-        <v>0.6216216216216216</v>
+        <v>0.8706896551724138</v>
       </c>
       <c r="L16" s="2">
-        <v>0.2387096774193548</v>
+        <v>0.2516268980477224</v>
       </c>
       <c r="M16" s="3">
-        <v>37</v>
+        <v>116</v>
       </c>
       <c r="N16" s="3">
-        <v>23</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="9:14">
@@ -2728,16 +2729,16 @@
         <v>8</v>
       </c>
       <c r="K17" s="2">
-        <v>0.1891891891891892</v>
+        <v>0.3269230769230769</v>
       </c>
       <c r="L17" s="2">
-        <v>0.3057851239669421</v>
+        <v>0.3959390862944163</v>
       </c>
       <c r="M17" s="3">
-        <v>37</v>
+        <v>156</v>
       </c>
       <c r="N17" s="3">
-        <v>7</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="9:14">
@@ -2748,16 +2749,16 @@
         <v>9</v>
       </c>
       <c r="K18" s="2">
-        <v>0.25</v>
+        <v>0.4864864864864865</v>
       </c>
       <c r="L18" s="2">
-        <v>0.3053435114503817</v>
+        <v>0.4195011337868481</v>
       </c>
       <c r="M18" s="3">
-        <v>40</v>
+        <v>185</v>
       </c>
       <c r="N18" s="3">
-        <v>10</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" spans="9:14">
@@ -2768,16 +2769,16 @@
         <v>10</v>
       </c>
       <c r="K19" s="2">
-        <v>0.2166666666666667</v>
+        <v>0.4943181818181818</v>
       </c>
       <c r="L19" s="2">
-        <v>0.3726708074534161</v>
+        <v>0.4074074074074074</v>
       </c>
       <c r="M19" s="3">
-        <v>60</v>
+        <v>176</v>
       </c>
       <c r="N19" s="3">
-        <v>13</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="9:14">
@@ -2788,16 +2789,16 @@
         <v>11</v>
       </c>
       <c r="K20" s="2">
-        <v>0.2857142857142857</v>
+        <v>0.4539473684210527</v>
       </c>
       <c r="L20" s="2">
-        <v>0.4294478527607362</v>
+        <v>0.3326039387308534</v>
       </c>
       <c r="M20" s="3">
-        <v>70</v>
+        <v>152</v>
       </c>
       <c r="N20" s="3">
-        <v>20</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="9:14">
@@ -2808,16 +2809,16 @@
         <v>12</v>
       </c>
       <c r="K21" s="2">
-        <v>0.2352941176470588</v>
+        <v>0.5135135135135135</v>
       </c>
       <c r="L21" s="2">
-        <v>0.3422818791946309</v>
+        <v>0.3363636363636364</v>
       </c>
       <c r="M21" s="3">
-        <v>51</v>
+        <v>148</v>
       </c>
       <c r="N21" s="3">
-        <v>12</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22" spans="9:14">
@@ -2828,16 +2829,16 @@
         <v>13</v>
       </c>
       <c r="K22" s="2">
-        <v>0.1551724137931035</v>
+        <v>0.4802631578947368</v>
       </c>
       <c r="L22" s="2">
-        <v>0.3892617449664429</v>
+        <v>0.3734643734643734</v>
       </c>
       <c r="M22" s="3">
-        <v>58</v>
+        <v>152</v>
       </c>
       <c r="N22" s="3">
-        <v>9</v>
+        <v>73</v>
       </c>
     </row>
     <row r="23" spans="9:14">
@@ -2848,16 +2849,16 @@
         <v>14</v>
       </c>
       <c r="K23" s="2">
-        <v>0.1964285714285714</v>
+        <v>0.4901960784313725</v>
       </c>
       <c r="L23" s="2">
-        <v>0.3809523809523809</v>
+        <v>0.3485193621867881</v>
       </c>
       <c r="M23" s="3">
-        <v>56</v>
+        <v>153</v>
       </c>
       <c r="N23" s="3">
-        <v>11</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24" spans="9:14">
@@ -2868,16 +2869,16 @@
         <v>15</v>
       </c>
       <c r="K24" s="2">
-        <v>0.2765957446808511</v>
+        <v>0.4796747967479675</v>
       </c>
       <c r="L24" s="2">
-        <v>0.3286713286713286</v>
+        <v>0.2992700729927008</v>
       </c>
       <c r="M24" s="3">
-        <v>47</v>
+        <v>123</v>
       </c>
       <c r="N24" s="3">
-        <v>13</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25" spans="9:14">
@@ -2888,16 +2889,16 @@
         <v>16</v>
       </c>
       <c r="K25" s="2">
-        <v>0.2549019607843137</v>
+        <v>0.456</v>
       </c>
       <c r="L25" s="2">
-        <v>0.3422818791946309</v>
+        <v>0.2955082742316785</v>
       </c>
       <c r="M25" s="3">
-        <v>51</v>
+        <v>125</v>
       </c>
       <c r="N25" s="3">
-        <v>13</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26" spans="9:14">
@@ -2908,16 +2909,16 @@
         <v>17</v>
       </c>
       <c r="K26" s="2">
-        <v>0.2916666666666667</v>
+        <v>0.5528455284552846</v>
       </c>
       <c r="L26" s="2">
-        <v>0.3380281690140845</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="M26" s="3">
-        <v>48</v>
+        <v>123</v>
       </c>
       <c r="N26" s="3">
-        <v>14</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" spans="9:14">
@@ -2928,16 +2929,16 @@
         <v>18</v>
       </c>
       <c r="K27" s="2">
-        <v>0.375</v>
+        <v>0.5</v>
       </c>
       <c r="L27" s="2">
-        <v>0.237037037037037</v>
+        <v>0.2645011600928074</v>
       </c>
       <c r="M27" s="3">
-        <v>32</v>
+        <v>114</v>
       </c>
       <c r="N27" s="3">
-        <v>12</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="9:14">
@@ -2948,16 +2949,16 @@
         <v>19</v>
       </c>
       <c r="K28" s="2">
-        <v>0.3333333333333333</v>
+        <v>0.5597014925373134</v>
       </c>
       <c r="L28" s="2">
-        <v>0.2635135135135135</v>
+        <v>0.2932166301969366</v>
       </c>
       <c r="M28" s="3">
-        <v>39</v>
+        <v>134</v>
       </c>
       <c r="N28" s="3">
-        <v>13</v>
+        <v>75</v>
       </c>
     </row>
     <row r="29" spans="9:14">
@@ -2968,16 +2969,16 @@
         <v>20</v>
       </c>
       <c r="K29" s="2">
-        <v>0.2380952380952381</v>
+        <v>0.5357142857142857</v>
       </c>
       <c r="L29" s="2">
-        <v>0.2709677419354839</v>
+        <v>0.3036876355748373</v>
       </c>
       <c r="M29" s="3">
-        <v>42</v>
+        <v>140</v>
       </c>
       <c r="N29" s="3">
-        <v>10</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="9:14">
@@ -2988,16 +2989,16 @@
         <v>8</v>
       </c>
       <c r="K30" s="2">
-        <v>0.07692307692307693</v>
+        <v>0</v>
       </c>
       <c r="L30" s="2">
-        <v>0.1074380165289256</v>
+        <v>0.1421319796954315</v>
       </c>
       <c r="M30" s="3">
-        <v>13</v>
+        <v>56</v>
       </c>
       <c r="N30" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="9:14">
@@ -3008,16 +3009,16 @@
         <v>9</v>
       </c>
       <c r="K31" s="2">
-        <v>0.08333333333333333</v>
+        <v>0.07954545454545454</v>
       </c>
       <c r="L31" s="2">
-        <v>0.0916030534351145</v>
+        <v>0.199546485260771</v>
       </c>
       <c r="M31" s="3">
-        <v>12</v>
+        <v>88</v>
       </c>
       <c r="N31" s="3">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32" spans="9:14">
@@ -3028,16 +3029,16 @@
         <v>10</v>
       </c>
       <c r="K32" s="2">
-        <v>0.1739130434782609</v>
+        <v>0.09174311926605505</v>
       </c>
       <c r="L32" s="2">
-        <v>0.1428571428571428</v>
+        <v>0.2523148148148148</v>
       </c>
       <c r="M32" s="3">
-        <v>23</v>
+        <v>109</v>
       </c>
       <c r="N32" s="3">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="9:14">
@@ -3048,16 +3049,16 @@
         <v>11</v>
       </c>
       <c r="K33" s="2">
-        <v>0.2</v>
+        <v>0.1458333333333333</v>
       </c>
       <c r="L33" s="2">
-        <v>0.2147239263803681</v>
+        <v>0.3150984682713348</v>
       </c>
       <c r="M33" s="3">
-        <v>35</v>
+        <v>144</v>
       </c>
       <c r="N33" s="3">
-        <v>7</v>
+        <v>21</v>
       </c>
     </row>
     <row r="34" spans="9:14">
@@ -3068,16 +3069,16 @@
         <v>12</v>
       </c>
       <c r="K34" s="2">
-        <v>0.1282051282051282</v>
+        <v>0.1052631578947368</v>
       </c>
       <c r="L34" s="2">
-        <v>0.261744966442953</v>
+        <v>0.3022727272727272</v>
       </c>
       <c r="M34" s="3">
-        <v>39</v>
+        <v>133</v>
       </c>
       <c r="N34" s="3">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="35" spans="9:14">
@@ -3088,16 +3089,16 @@
         <v>13</v>
       </c>
       <c r="K35" s="2">
-        <v>0.1627906976744186</v>
+        <v>0.1395348837209302</v>
       </c>
       <c r="L35" s="2">
-        <v>0.2885906040268457</v>
+        <v>0.316953316953317</v>
       </c>
       <c r="M35" s="3">
-        <v>43</v>
+        <v>129</v>
       </c>
       <c r="N35" s="3">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="36" spans="9:14">
@@ -3108,16 +3109,16 @@
         <v>14</v>
       </c>
       <c r="K36" s="2">
-        <v>0.16</v>
+        <v>0.1458333333333333</v>
       </c>
       <c r="L36" s="2">
-        <v>0.3401360544217687</v>
+        <v>0.3280182232346242</v>
       </c>
       <c r="M36" s="3">
-        <v>50</v>
+        <v>144</v>
       </c>
       <c r="N36" s="3">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="37" spans="9:14">
@@ -3128,16 +3129,16 @@
         <v>15</v>
       </c>
       <c r="K37" s="2">
-        <v>0.09836065573770492</v>
+        <v>0.1059602649006623</v>
       </c>
       <c r="L37" s="2">
-        <v>0.4265734265734266</v>
+        <v>0.3673965936739659</v>
       </c>
       <c r="M37" s="3">
-        <v>61</v>
+        <v>151</v>
       </c>
       <c r="N37" s="3">
-        <v>6</v>
+        <v>16</v>
       </c>
     </row>
     <row r="38" spans="9:14">
@@ -3148,16 +3149,16 @@
         <v>16</v>
       </c>
       <c r="K38" s="2">
-        <v>0.1857142857142857</v>
+        <v>0.09580838323353294</v>
       </c>
       <c r="L38" s="2">
-        <v>0.4697986577181208</v>
+        <v>0.3947990543735225</v>
       </c>
       <c r="M38" s="3">
-        <v>70</v>
+        <v>167</v>
       </c>
       <c r="N38" s="3">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="39" spans="9:14">
@@ -3168,16 +3169,16 @@
         <v>17</v>
       </c>
       <c r="K39" s="2">
-        <v>0.180327868852459</v>
+        <v>0.09659090909090909</v>
       </c>
       <c r="L39" s="2">
-        <v>0.4295774647887324</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="M39" s="3">
-        <v>61</v>
+        <v>176</v>
       </c>
       <c r="N39" s="3">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
     <row r="40" spans="9:14">
@@ -3188,16 +3189,16 @@
         <v>18</v>
       </c>
       <c r="K40" s="2">
-        <v>0.07792207792207792</v>
+        <v>0.1047120418848168</v>
       </c>
       <c r="L40" s="2">
-        <v>0.5703703703703704</v>
+        <v>0.4431554524361949</v>
       </c>
       <c r="M40" s="3">
-        <v>77</v>
+        <v>191</v>
       </c>
       <c r="N40" s="3">
-        <v>6</v>
+        <v>20</v>
       </c>
     </row>
     <row r="41" spans="9:14">
@@ -3208,16 +3209,16 @@
         <v>19</v>
       </c>
       <c r="K41" s="2">
-        <v>0.1267605633802817</v>
+        <v>0.1170212765957447</v>
       </c>
       <c r="L41" s="2">
-        <v>0.4797297297297297</v>
+        <v>0.4113785557986871</v>
       </c>
       <c r="M41" s="3">
-        <v>71</v>
+        <v>188</v>
       </c>
       <c r="N41" s="3">
-        <v>9</v>
+        <v>22</v>
       </c>
     </row>
     <row r="42" spans="9:14">
@@ -3228,16 +3229,16 @@
         <v>20</v>
       </c>
       <c r="K42" s="2">
-        <v>0.07894736842105263</v>
+        <v>0.07804878048780488</v>
       </c>
       <c r="L42" s="2">
-        <v>0.4903225806451613</v>
+        <v>0.4446854663774403</v>
       </c>
       <c r="M42" s="3">
-        <v>76</v>
+        <v>205</v>
       </c>
       <c r="N42" s="3">
-        <v>6</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -3252,7 +3253,8 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.7109375" style="1" customWidth="1"/>
-    <col min="2" max="3" width="21.7109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="21.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" style="1" customWidth="1"/>
     <col min="4" max="4" width="21.7109375" style="2" customWidth="1"/>
     <col min="5" max="5" width="20.7109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.7109375" style="1" customWidth="1"/>
@@ -3311,22 +3313,22 @@
         <v>0</v>
       </c>
       <c r="B4" s="1">
-        <v>-0.5174374683146535</v>
+        <v>0.9502345014917034</v>
       </c>
       <c r="C4" s="1">
-        <v>3.203767666961591</v>
+        <v>8.014037340297495</v>
       </c>
       <c r="D4" s="2">
-        <v>0.5942947702060222</v>
+        <v>0.8767268862911796</v>
       </c>
       <c r="E4" s="1">
-        <v>0.3333333333333333</v>
+        <v>0.3334514528703048</v>
       </c>
       <c r="F4" s="1">
-        <v>3155000</v>
+        <v>9410000</v>
       </c>
       <c r="G4" s="1">
-        <v>1875000</v>
+        <v>8250000</v>
       </c>
       <c r="I4" s="1">
         <v>0</v>
@@ -3335,16 +3337,16 @@
         <v>8</v>
       </c>
       <c r="K4" s="2">
-        <v>0.5211267605633803</v>
+        <v>0.8131868131868132</v>
       </c>
       <c r="L4" s="1">
-        <v>0.5867768595041323</v>
+        <v>0.4619289340101523</v>
       </c>
       <c r="M4" s="1">
-        <v>355000</v>
+        <v>910000</v>
       </c>
       <c r="N4" s="1">
-        <v>185000</v>
+        <v>740000</v>
       </c>
     </row>
     <row r="5" spans="1:14">
@@ -3352,22 +3354,22 @@
         <v>1</v>
       </c>
       <c r="B5" s="1">
-        <v>-1.135530545938961</v>
+        <v>-1.043918035281563</v>
       </c>
       <c r="C5" s="1">
-        <v>-0.5181460438793203</v>
+        <v>0.9500194933372372</v>
       </c>
       <c r="D5" s="2">
-        <v>0.248811410459588</v>
+        <v>0.4848484848484849</v>
       </c>
       <c r="E5" s="1">
-        <v>0.3333333333333333</v>
+        <v>0.3332742735648476</v>
       </c>
       <c r="F5" s="1">
-        <v>3155000</v>
+        <v>9405000</v>
       </c>
       <c r="G5" s="1">
-        <v>785000</v>
+        <v>4560000</v>
       </c>
       <c r="I5" s="1">
         <v>0</v>
@@ -3376,16 +3378,16 @@
         <v>9</v>
       </c>
       <c r="K5" s="2">
-        <v>0.5189873417721519</v>
+        <v>0.9047619047619048</v>
       </c>
       <c r="L5" s="1">
-        <v>0.6030534351145038</v>
+        <v>0.3809523809523809</v>
       </c>
       <c r="M5" s="1">
-        <v>395000</v>
+        <v>840000</v>
       </c>
       <c r="N5" s="1">
-        <v>205000</v>
+        <v>760000</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -3393,22 +3395,22 @@
         <v>2</v>
       </c>
       <c r="B6" s="1">
-        <v>-2.435104178233598</v>
+        <v>-10.8317280747611</v>
       </c>
       <c r="C6" s="1">
-        <v>-1.136348485150166</v>
+        <v>-1.045108577584102</v>
       </c>
       <c r="D6" s="2">
-        <v>0.133122028526149</v>
+        <v>0.1052631578947368</v>
       </c>
       <c r="E6" s="1">
-        <v>0.3333333333333333</v>
+        <v>0.3332742735648476</v>
       </c>
       <c r="F6" s="1">
-        <v>3155000</v>
+        <v>9405000</v>
       </c>
       <c r="G6" s="1">
-        <v>420000</v>
+        <v>990000</v>
       </c>
       <c r="I6" s="1">
         <v>0</v>
@@ -3417,16 +3419,16 @@
         <v>10</v>
       </c>
       <c r="K6" s="2">
-        <v>0.6410256410256411</v>
+        <v>0.9047619047619048</v>
       </c>
       <c r="L6" s="1">
-        <v>0.484472049689441</v>
+        <v>0.3402777777777778</v>
       </c>
       <c r="M6" s="1">
-        <v>390000</v>
+        <v>735000</v>
       </c>
       <c r="N6" s="1">
-        <v>250000</v>
+        <v>665000</v>
       </c>
     </row>
     <row r="7" spans="1:14">
@@ -3437,16 +3439,16 @@
         <v>11</v>
       </c>
       <c r="K7" s="2">
-        <v>0.5689655172413793</v>
+        <v>0.937888198757764</v>
       </c>
       <c r="L7" s="1">
-        <v>0.3558282208588957</v>
+        <v>0.3522975929978118</v>
       </c>
       <c r="M7" s="1">
-        <v>290000</v>
+        <v>805000</v>
       </c>
       <c r="N7" s="1">
-        <v>165000</v>
+        <v>755000</v>
       </c>
     </row>
     <row r="8" spans="1:14">
@@ -3457,16 +3459,16 @@
         <v>12</v>
       </c>
       <c r="K8" s="2">
-        <v>0.6949152542372882</v>
+        <v>0.9182389937106918</v>
       </c>
       <c r="L8" s="1">
-        <v>0.3959731543624161</v>
+        <v>0.3613636363636364</v>
       </c>
       <c r="M8" s="1">
-        <v>295000</v>
+        <v>795000</v>
       </c>
       <c r="N8" s="1">
-        <v>205000</v>
+        <v>730000</v>
       </c>
     </row>
     <row r="9" spans="1:14">
@@ -3477,16 +3479,16 @@
         <v>13</v>
       </c>
       <c r="K9" s="2">
-        <v>0.7083333333333334</v>
+        <v>0.9047619047619048</v>
       </c>
       <c r="L9" s="1">
-        <v>0.3221476510067114</v>
+        <v>0.3095823095823096</v>
       </c>
       <c r="M9" s="1">
-        <v>240000</v>
+        <v>630000</v>
       </c>
       <c r="N9" s="1">
-        <v>170000</v>
+        <v>570000</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -3497,16 +3499,16 @@
         <v>14</v>
       </c>
       <c r="K10" s="2">
-        <v>0.6341463414634146</v>
+        <v>0.8873239436619719</v>
       </c>
       <c r="L10" s="1">
-        <v>0.2789115646258503</v>
+        <v>0.3234624145785877</v>
       </c>
       <c r="M10" s="1">
-        <v>205000</v>
+        <v>710000</v>
       </c>
       <c r="N10" s="1">
-        <v>130000</v>
+        <v>630000</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -3517,16 +3519,16 @@
         <v>15</v>
       </c>
       <c r="K11" s="2">
-        <v>0.6571428571428571</v>
+        <v>0.8686131386861314</v>
       </c>
       <c r="L11" s="1">
-        <v>0.2447552447552448</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="M11" s="1">
-        <v>175000</v>
+        <v>685000</v>
       </c>
       <c r="N11" s="1">
-        <v>115000</v>
+        <v>595000</v>
       </c>
     </row>
     <row r="12" spans="1:14">
@@ -3537,16 +3539,16 @@
         <v>16</v>
       </c>
       <c r="K12" s="2">
-        <v>0.3928571428571428</v>
+        <v>0.8625954198473282</v>
       </c>
       <c r="L12" s="1">
-        <v>0.1879194630872483</v>
+        <v>0.3096926713947991</v>
       </c>
       <c r="M12" s="1">
-        <v>140000</v>
+        <v>655000</v>
       </c>
       <c r="N12" s="1">
-        <v>55000</v>
+        <v>565000</v>
       </c>
     </row>
     <row r="13" spans="1:14">
@@ -3557,16 +3559,16 @@
         <v>17</v>
       </c>
       <c r="K13" s="2">
-        <v>0.6363636363636364</v>
+        <v>0.881578947368421</v>
       </c>
       <c r="L13" s="1">
-        <v>0.2323943661971831</v>
+        <v>0.3370288248337029</v>
       </c>
       <c r="M13" s="1">
-        <v>165000</v>
+        <v>760000</v>
       </c>
       <c r="N13" s="1">
-        <v>105000</v>
+        <v>670000</v>
       </c>
     </row>
     <row r="14" spans="1:14">
@@ -3577,16 +3579,16 @@
         <v>18</v>
       </c>
       <c r="K14" s="2">
-        <v>0.5384615384615384</v>
+        <v>0.8095238095238095</v>
       </c>
       <c r="L14" s="1">
-        <v>0.1925925925925926</v>
+        <v>0.2923433874709977</v>
       </c>
       <c r="M14" s="1">
-        <v>130000</v>
+        <v>630000</v>
       </c>
       <c r="N14" s="1">
-        <v>70000</v>
+        <v>510000</v>
       </c>
     </row>
     <row r="15" spans="1:14">
@@ -3597,16 +3599,16 @@
         <v>19</v>
       </c>
       <c r="K15" s="2">
-        <v>0.5526315789473685</v>
+        <v>0.8222222222222222</v>
       </c>
       <c r="L15" s="1">
-        <v>0.2567567567567567</v>
+        <v>0.2954048140043763</v>
       </c>
       <c r="M15" s="1">
-        <v>190000</v>
+        <v>675000</v>
       </c>
       <c r="N15" s="1">
-        <v>105000</v>
+        <v>555000</v>
       </c>
     </row>
     <row r="16" spans="1:14">
@@ -3617,16 +3619,16 @@
         <v>20</v>
       </c>
       <c r="K16" s="2">
-        <v>0.6216216216216216</v>
+        <v>0.8706896551724138</v>
       </c>
       <c r="L16" s="1">
-        <v>0.2387096774193548</v>
+        <v>0.2516268980477224</v>
       </c>
       <c r="M16" s="1">
-        <v>185000</v>
+        <v>580000</v>
       </c>
       <c r="N16" s="1">
-        <v>115000</v>
+        <v>505000</v>
       </c>
     </row>
     <row r="17" spans="9:14">
@@ -3637,16 +3639,16 @@
         <v>8</v>
       </c>
       <c r="K17" s="2">
-        <v>0.1891891891891892</v>
+        <v>0.3269230769230769</v>
       </c>
       <c r="L17" s="1">
-        <v>0.3057851239669421</v>
+        <v>0.3959390862944163</v>
       </c>
       <c r="M17" s="1">
-        <v>185000</v>
+        <v>780000</v>
       </c>
       <c r="N17" s="1">
-        <v>35000</v>
+        <v>255000</v>
       </c>
     </row>
     <row r="18" spans="9:14">
@@ -3657,16 +3659,16 @@
         <v>9</v>
       </c>
       <c r="K18" s="2">
-        <v>0.25</v>
+        <v>0.4864864864864865</v>
       </c>
       <c r="L18" s="1">
-        <v>0.3053435114503817</v>
+        <v>0.4195011337868481</v>
       </c>
       <c r="M18" s="1">
-        <v>200000</v>
+        <v>925000</v>
       </c>
       <c r="N18" s="1">
-        <v>50000</v>
+        <v>450000</v>
       </c>
     </row>
     <row r="19" spans="9:14">
@@ -3677,16 +3679,16 @@
         <v>10</v>
       </c>
       <c r="K19" s="2">
-        <v>0.2166666666666667</v>
+        <v>0.4943181818181818</v>
       </c>
       <c r="L19" s="1">
-        <v>0.3726708074534161</v>
+        <v>0.4074074074074074</v>
       </c>
       <c r="M19" s="1">
-        <v>300000</v>
+        <v>880000</v>
       </c>
       <c r="N19" s="1">
-        <v>65000</v>
+        <v>435000</v>
       </c>
     </row>
     <row r="20" spans="9:14">
@@ -3697,16 +3699,16 @@
         <v>11</v>
       </c>
       <c r="K20" s="2">
-        <v>0.2857142857142857</v>
+        <v>0.4539473684210527</v>
       </c>
       <c r="L20" s="1">
-        <v>0.4294478527607362</v>
+        <v>0.3326039387308534</v>
       </c>
       <c r="M20" s="1">
-        <v>350000</v>
+        <v>760000</v>
       </c>
       <c r="N20" s="1">
-        <v>100000</v>
+        <v>345000</v>
       </c>
     </row>
     <row r="21" spans="9:14">
@@ -3717,16 +3719,16 @@
         <v>12</v>
       </c>
       <c r="K21" s="2">
-        <v>0.2352941176470588</v>
+        <v>0.5135135135135135</v>
       </c>
       <c r="L21" s="1">
-        <v>0.3422818791946309</v>
+        <v>0.3363636363636364</v>
       </c>
       <c r="M21" s="1">
-        <v>255000</v>
+        <v>740000</v>
       </c>
       <c r="N21" s="1">
-        <v>60000</v>
+        <v>380000</v>
       </c>
     </row>
     <row r="22" spans="9:14">
@@ -3737,16 +3739,16 @@
         <v>13</v>
       </c>
       <c r="K22" s="2">
-        <v>0.1551724137931035</v>
+        <v>0.4802631578947368</v>
       </c>
       <c r="L22" s="1">
-        <v>0.3892617449664429</v>
+        <v>0.3734643734643734</v>
       </c>
       <c r="M22" s="1">
-        <v>290000</v>
+        <v>760000</v>
       </c>
       <c r="N22" s="1">
-        <v>45000</v>
+        <v>365000</v>
       </c>
     </row>
     <row r="23" spans="9:14">
@@ -3757,16 +3759,16 @@
         <v>14</v>
       </c>
       <c r="K23" s="2">
-        <v>0.1964285714285714</v>
+        <v>0.4901960784313725</v>
       </c>
       <c r="L23" s="1">
-        <v>0.3809523809523809</v>
+        <v>0.3485193621867881</v>
       </c>
       <c r="M23" s="1">
-        <v>280000</v>
+        <v>765000</v>
       </c>
       <c r="N23" s="1">
-        <v>55000</v>
+        <v>375000</v>
       </c>
     </row>
     <row r="24" spans="9:14">
@@ -3777,16 +3779,16 @@
         <v>15</v>
       </c>
       <c r="K24" s="2">
-        <v>0.2765957446808511</v>
+        <v>0.4796747967479675</v>
       </c>
       <c r="L24" s="1">
-        <v>0.3286713286713286</v>
+        <v>0.2992700729927008</v>
       </c>
       <c r="M24" s="1">
-        <v>235000</v>
+        <v>615000</v>
       </c>
       <c r="N24" s="1">
-        <v>65000</v>
+        <v>295000</v>
       </c>
     </row>
     <row r="25" spans="9:14">
@@ -3797,16 +3799,16 @@
         <v>16</v>
       </c>
       <c r="K25" s="2">
-        <v>0.2549019607843137</v>
+        <v>0.456</v>
       </c>
       <c r="L25" s="1">
-        <v>0.3422818791946309</v>
+        <v>0.2955082742316785</v>
       </c>
       <c r="M25" s="1">
-        <v>255000</v>
+        <v>625000</v>
       </c>
       <c r="N25" s="1">
-        <v>65000</v>
+        <v>285000</v>
       </c>
     </row>
     <row r="26" spans="9:14">
@@ -3817,16 +3819,16 @@
         <v>17</v>
       </c>
       <c r="K26" s="2">
-        <v>0.2916666666666667</v>
+        <v>0.5528455284552846</v>
       </c>
       <c r="L26" s="1">
-        <v>0.3380281690140845</v>
+        <v>0.2727272727272727</v>
       </c>
       <c r="M26" s="1">
-        <v>240000</v>
+        <v>615000</v>
       </c>
       <c r="N26" s="1">
-        <v>70000</v>
+        <v>340000</v>
       </c>
     </row>
     <row r="27" spans="9:14">
@@ -3837,16 +3839,16 @@
         <v>18</v>
       </c>
       <c r="K27" s="2">
-        <v>0.375</v>
+        <v>0.5</v>
       </c>
       <c r="L27" s="1">
-        <v>0.237037037037037</v>
+        <v>0.2645011600928074</v>
       </c>
       <c r="M27" s="1">
-        <v>160000</v>
+        <v>570000</v>
       </c>
       <c r="N27" s="1">
-        <v>60000</v>
+        <v>285000</v>
       </c>
     </row>
     <row r="28" spans="9:14">
@@ -3857,16 +3859,16 @@
         <v>19</v>
       </c>
       <c r="K28" s="2">
-        <v>0.3333333333333333</v>
+        <v>0.5597014925373134</v>
       </c>
       <c r="L28" s="1">
-        <v>0.2635135135135135</v>
+        <v>0.2932166301969366</v>
       </c>
       <c r="M28" s="1">
-        <v>195000</v>
+        <v>670000</v>
       </c>
       <c r="N28" s="1">
-        <v>65000</v>
+        <v>375000</v>
       </c>
     </row>
     <row r="29" spans="9:14">
@@ -3877,16 +3879,16 @@
         <v>20</v>
       </c>
       <c r="K29" s="2">
-        <v>0.2380952380952381</v>
+        <v>0.5357142857142857</v>
       </c>
       <c r="L29" s="1">
-        <v>0.2709677419354839</v>
+        <v>0.3036876355748373</v>
       </c>
       <c r="M29" s="1">
-        <v>210000</v>
+        <v>700000</v>
       </c>
       <c r="N29" s="1">
-        <v>50000</v>
+        <v>375000</v>
       </c>
     </row>
     <row r="30" spans="9:14">
@@ -3897,16 +3899,16 @@
         <v>8</v>
       </c>
       <c r="K30" s="2">
-        <v>0.07692307692307693</v>
+        <v>0</v>
       </c>
       <c r="L30" s="1">
-        <v>0.1074380165289256</v>
+        <v>0.1421319796954315</v>
       </c>
       <c r="M30" s="1">
-        <v>65000</v>
+        <v>280000</v>
       </c>
       <c r="N30" s="1">
-        <v>5000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="9:14">
@@ -3917,16 +3919,16 @@
         <v>9</v>
       </c>
       <c r="K31" s="2">
-        <v>0.08333333333333333</v>
+        <v>0.07954545454545454</v>
       </c>
       <c r="L31" s="1">
-        <v>0.0916030534351145</v>
+        <v>0.199546485260771</v>
       </c>
       <c r="M31" s="1">
-        <v>60000</v>
+        <v>440000</v>
       </c>
       <c r="N31" s="1">
-        <v>5000</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="32" spans="9:14">
@@ -3937,16 +3939,16 @@
         <v>10</v>
       </c>
       <c r="K32" s="2">
-        <v>0.1739130434782609</v>
+        <v>0.09174311926605505</v>
       </c>
       <c r="L32" s="1">
-        <v>0.1428571428571428</v>
+        <v>0.2523148148148148</v>
       </c>
       <c r="M32" s="1">
-        <v>115000</v>
+        <v>545000</v>
       </c>
       <c r="N32" s="1">
-        <v>20000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="33" spans="9:14">
@@ -3957,16 +3959,16 @@
         <v>11</v>
       </c>
       <c r="K33" s="2">
-        <v>0.2</v>
+        <v>0.1458333333333333</v>
       </c>
       <c r="L33" s="1">
-        <v>0.2147239263803681</v>
+        <v>0.3150984682713348</v>
       </c>
       <c r="M33" s="1">
-        <v>175000</v>
+        <v>720000</v>
       </c>
       <c r="N33" s="1">
-        <v>35000</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="34" spans="9:14">
@@ -3977,16 +3979,16 @@
         <v>12</v>
       </c>
       <c r="K34" s="2">
-        <v>0.1282051282051282</v>
+        <v>0.1052631578947368</v>
       </c>
       <c r="L34" s="1">
-        <v>0.261744966442953</v>
+        <v>0.3022727272727272</v>
       </c>
       <c r="M34" s="1">
-        <v>195000</v>
+        <v>665000</v>
       </c>
       <c r="N34" s="1">
-        <v>25000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="35" spans="9:14">
@@ -3997,16 +3999,16 @@
         <v>13</v>
       </c>
       <c r="K35" s="2">
-        <v>0.1627906976744186</v>
+        <v>0.1395348837209302</v>
       </c>
       <c r="L35" s="1">
-        <v>0.2885906040268457</v>
+        <v>0.316953316953317</v>
       </c>
       <c r="M35" s="1">
-        <v>215000</v>
+        <v>645000</v>
       </c>
       <c r="N35" s="1">
-        <v>35000</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="36" spans="9:14">
@@ -4017,16 +4019,16 @@
         <v>14</v>
       </c>
       <c r="K36" s="2">
-        <v>0.16</v>
+        <v>0.1458333333333333</v>
       </c>
       <c r="L36" s="1">
-        <v>0.3401360544217687</v>
+        <v>0.3280182232346242</v>
       </c>
       <c r="M36" s="1">
-        <v>250000</v>
+        <v>720000</v>
       </c>
       <c r="N36" s="1">
-        <v>40000</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="37" spans="9:14">
@@ -4037,16 +4039,16 @@
         <v>15</v>
       </c>
       <c r="K37" s="2">
-        <v>0.09836065573770492</v>
+        <v>0.1059602649006623</v>
       </c>
       <c r="L37" s="1">
-        <v>0.4265734265734266</v>
+        <v>0.3673965936739659</v>
       </c>
       <c r="M37" s="1">
-        <v>305000</v>
+        <v>755000</v>
       </c>
       <c r="N37" s="1">
-        <v>30000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="38" spans="9:14">
@@ -4057,16 +4059,16 @@
         <v>16</v>
       </c>
       <c r="K38" s="2">
-        <v>0.1857142857142857</v>
+        <v>0.09580838323353294</v>
       </c>
       <c r="L38" s="1">
-        <v>0.4697986577181208</v>
+        <v>0.3947990543735225</v>
       </c>
       <c r="M38" s="1">
-        <v>350000</v>
+        <v>835000</v>
       </c>
       <c r="N38" s="1">
-        <v>65000</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="39" spans="9:14">
@@ -4077,16 +4079,16 @@
         <v>17</v>
       </c>
       <c r="K39" s="2">
-        <v>0.180327868852459</v>
+        <v>0.09659090909090909</v>
       </c>
       <c r="L39" s="1">
-        <v>0.4295774647887324</v>
+        <v>0.3902439024390244</v>
       </c>
       <c r="M39" s="1">
-        <v>305000</v>
+        <v>880000</v>
       </c>
       <c r="N39" s="1">
-        <v>55000</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="40" spans="9:14">
@@ -4097,16 +4099,16 @@
         <v>18</v>
       </c>
       <c r="K40" s="2">
-        <v>0.07792207792207792</v>
+        <v>0.1047120418848168</v>
       </c>
       <c r="L40" s="1">
-        <v>0.5703703703703704</v>
+        <v>0.4431554524361949</v>
       </c>
       <c r="M40" s="1">
-        <v>385000</v>
+        <v>955000</v>
       </c>
       <c r="N40" s="1">
-        <v>30000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="41" spans="9:14">
@@ -4117,16 +4119,16 @@
         <v>19</v>
       </c>
       <c r="K41" s="2">
-        <v>0.1267605633802817</v>
+        <v>0.1170212765957447</v>
       </c>
       <c r="L41" s="1">
-        <v>0.4797297297297297</v>
+        <v>0.4113785557986871</v>
       </c>
       <c r="M41" s="1">
-        <v>355000</v>
+        <v>940000</v>
       </c>
       <c r="N41" s="1">
-        <v>45000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="42" spans="9:14">
@@ -4137,16 +4139,16 @@
         <v>20</v>
       </c>
       <c r="K42" s="2">
-        <v>0.07894736842105263</v>
+        <v>0.07804878048780488</v>
       </c>
       <c r="L42" s="1">
-        <v>0.4903225806451613</v>
+        <v>0.4446854663774403</v>
       </c>
       <c r="M42" s="1">
-        <v>380000</v>
+        <v>1025000</v>
       </c>
       <c r="N42" s="1">
-        <v>30000</v>
+        <v>80000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>